<commit_message>
annotation sheet example small edit
</commit_message>
<xml_diff>
--- a/example_data/annotation-sheet annotator-1.xlsx
+++ b/example_data/annotation-sheet annotator-1.xlsx
@@ -1,17 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dsouzaj\Desktop\Datasets\ALD-E-ImageMiner\example_data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7520"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="paper 1" sheetId="1" r:id="rId4"/>
+    <sheet name="paper 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
   <si>
     <t>prolific ID</t>
   </si>
@@ -412,48 +420,63 @@
   <si>
     <t>https://github.com/sciknoworg/ALD-E-ImageMiner/blob/main/example_data/1/images/figures/figure_15.summary.txt</t>
   </si>
+  <si>
+    <t>Overall Comments</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="5">
@@ -461,7 +484,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -483,56 +506,47 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -722,31 +736,34 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:AC16"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="16.25"/>
-    <col customWidth="1" min="2" max="2" width="19.38"/>
-    <col customWidth="1" min="3" max="3" width="27.13"/>
-    <col customWidth="1" min="4" max="4" width="16.25"/>
-    <col customWidth="1" min="5" max="5" width="15.63"/>
-    <col customWidth="1" min="6" max="6" width="21.38"/>
-    <col customWidth="1" min="7" max="8" width="22.0"/>
-    <col customWidth="1" min="9" max="9" width="15.38"/>
-    <col customWidth="1" min="10" max="10" width="15.13"/>
-    <col customWidth="1" min="11" max="11" width="24.63"/>
-    <col customWidth="1" min="12" max="12" width="42.25"/>
-    <col customWidth="1" min="13" max="13" width="18.75"/>
+    <col min="1" max="1" width="16.26953125" customWidth="1"/>
+    <col min="2" max="2" width="19.36328125" customWidth="1"/>
+    <col min="3" max="3" width="27.08984375" customWidth="1"/>
+    <col min="4" max="4" width="16.26953125" customWidth="1"/>
+    <col min="5" max="5" width="15.6328125" customWidth="1"/>
+    <col min="6" max="6" width="21.36328125" customWidth="1"/>
+    <col min="7" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="15.36328125" customWidth="1"/>
+    <col min="10" max="10" width="15.08984375" customWidth="1"/>
+    <col min="11" max="11" width="24.6328125" customWidth="1"/>
+    <col min="12" max="12" width="42.26953125" customWidth="1"/>
+    <col min="13" max="13" width="18.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:29" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -831,8 +848,11 @@
       <c r="AB1" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2">
+      <c r="AC1" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="3" t="s">
         <v>28</v>
@@ -856,7 +876,7 @@
       </c>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" ht="30.75" customHeight="1">
+    <row r="3" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="3" t="s">
@@ -879,7 +899,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" ht="26.25" customHeight="1">
+    <row r="4" spans="1:29" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="3" t="s">
@@ -905,7 +925,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="3" t="s">
@@ -928,7 +948,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="3" t="s">
@@ -954,7 +974,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="3" t="s">
@@ -980,7 +1000,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
       <c r="B8" s="7"/>
       <c r="C8" s="8" t="s">
@@ -1003,7 +1023,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="3" t="s">
@@ -1026,7 +1046,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="3" t="s">
@@ -1052,7 +1072,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="3" t="s">
@@ -1077,7 +1097,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="3" t="s">
@@ -1102,7 +1122,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="3" t="s">
@@ -1121,7 +1141,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="3" t="s">
@@ -1146,7 +1166,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="3" t="s">
@@ -1168,7 +1188,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="3" t="s">
@@ -1192,68 +1212,68 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="B2"/>
-    <hyperlink r:id="rId2" ref="C2"/>
-    <hyperlink r:id="rId3" ref="E2"/>
-    <hyperlink r:id="rId4" ref="H2"/>
-    <hyperlink r:id="rId5" ref="J2"/>
-    <hyperlink r:id="rId6" ref="C3"/>
-    <hyperlink r:id="rId7" ref="E3"/>
-    <hyperlink r:id="rId8" ref="H3"/>
-    <hyperlink r:id="rId9" ref="J3"/>
-    <hyperlink r:id="rId10" ref="C4"/>
-    <hyperlink r:id="rId11" ref="E4"/>
-    <hyperlink r:id="rId12" ref="H4"/>
-    <hyperlink r:id="rId13" ref="J4"/>
-    <hyperlink r:id="rId14" ref="C5"/>
-    <hyperlink r:id="rId15" ref="E5"/>
-    <hyperlink r:id="rId16" ref="H5"/>
-    <hyperlink r:id="rId17" ref="J5"/>
-    <hyperlink r:id="rId18" ref="C6"/>
-    <hyperlink r:id="rId19" ref="E6"/>
-    <hyperlink r:id="rId20" ref="H6"/>
-    <hyperlink r:id="rId21" ref="J6"/>
-    <hyperlink r:id="rId22" ref="C7"/>
-    <hyperlink r:id="rId23" ref="E7"/>
-    <hyperlink r:id="rId24" ref="H7"/>
-    <hyperlink r:id="rId25" ref="J7"/>
-    <hyperlink r:id="rId26" ref="C8"/>
-    <hyperlink r:id="rId27" ref="E8"/>
-    <hyperlink r:id="rId28" ref="H8"/>
-    <hyperlink r:id="rId29" ref="J8"/>
-    <hyperlink r:id="rId30" ref="C9"/>
-    <hyperlink r:id="rId31" ref="E9"/>
-    <hyperlink r:id="rId32" ref="H9"/>
-    <hyperlink r:id="rId33" ref="J9"/>
-    <hyperlink r:id="rId34" ref="C10"/>
-    <hyperlink r:id="rId35" ref="E10"/>
-    <hyperlink r:id="rId36" ref="H10"/>
-    <hyperlink r:id="rId37" ref="J10"/>
-    <hyperlink r:id="rId38" ref="C11"/>
-    <hyperlink r:id="rId39" ref="E11"/>
-    <hyperlink r:id="rId40" ref="H11"/>
-    <hyperlink r:id="rId41" ref="J11"/>
-    <hyperlink r:id="rId42" ref="C12"/>
-    <hyperlink r:id="rId43" ref="E12"/>
-    <hyperlink r:id="rId44" ref="H12"/>
-    <hyperlink r:id="rId45" ref="J12"/>
-    <hyperlink r:id="rId46" ref="C13"/>
-    <hyperlink r:id="rId47" ref="E13"/>
-    <hyperlink r:id="rId48" ref="H13"/>
-    <hyperlink r:id="rId49" ref="J13"/>
-    <hyperlink r:id="rId50" ref="C14"/>
-    <hyperlink r:id="rId51" ref="E14"/>
-    <hyperlink r:id="rId52" ref="H14"/>
-    <hyperlink r:id="rId53" ref="J14"/>
-    <hyperlink r:id="rId54" ref="C15"/>
-    <hyperlink r:id="rId55" ref="E15"/>
-    <hyperlink r:id="rId56" ref="H15"/>
-    <hyperlink r:id="rId57" ref="J15"/>
-    <hyperlink r:id="rId58" ref="C16"/>
-    <hyperlink r:id="rId59" ref="E16"/>
-    <hyperlink r:id="rId60" ref="H16"/>
-    <hyperlink r:id="rId61" ref="J16"/>
+    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="C2" r:id="rId2"/>
+    <hyperlink ref="E2" r:id="rId3"/>
+    <hyperlink ref="H2" r:id="rId4"/>
+    <hyperlink ref="J2" r:id="rId5"/>
+    <hyperlink ref="C3" r:id="rId6"/>
+    <hyperlink ref="E3" r:id="rId7"/>
+    <hyperlink ref="H3" r:id="rId8"/>
+    <hyperlink ref="J3" r:id="rId9"/>
+    <hyperlink ref="C4" r:id="rId10"/>
+    <hyperlink ref="E4" r:id="rId11"/>
+    <hyperlink ref="H4" r:id="rId12"/>
+    <hyperlink ref="J4" r:id="rId13"/>
+    <hyperlink ref="C5" r:id="rId14"/>
+    <hyperlink ref="E5" r:id="rId15"/>
+    <hyperlink ref="H5" r:id="rId16"/>
+    <hyperlink ref="J5" r:id="rId17"/>
+    <hyperlink ref="C6" r:id="rId18"/>
+    <hyperlink ref="E6" r:id="rId19"/>
+    <hyperlink ref="H6" r:id="rId20"/>
+    <hyperlink ref="J6" r:id="rId21"/>
+    <hyperlink ref="C7" r:id="rId22"/>
+    <hyperlink ref="E7" r:id="rId23"/>
+    <hyperlink ref="H7" r:id="rId24"/>
+    <hyperlink ref="J7" r:id="rId25"/>
+    <hyperlink ref="C8" r:id="rId26"/>
+    <hyperlink ref="E8" r:id="rId27"/>
+    <hyperlink ref="H8" r:id="rId28"/>
+    <hyperlink ref="J8" r:id="rId29"/>
+    <hyperlink ref="C9" r:id="rId30"/>
+    <hyperlink ref="E9" r:id="rId31"/>
+    <hyperlink ref="H9" r:id="rId32"/>
+    <hyperlink ref="J9" r:id="rId33"/>
+    <hyperlink ref="C10" r:id="rId34"/>
+    <hyperlink ref="E10" r:id="rId35"/>
+    <hyperlink ref="H10" r:id="rId36"/>
+    <hyperlink ref="J10" r:id="rId37"/>
+    <hyperlink ref="C11" r:id="rId38"/>
+    <hyperlink ref="E11" r:id="rId39"/>
+    <hyperlink ref="H11" r:id="rId40"/>
+    <hyperlink ref="J11" r:id="rId41"/>
+    <hyperlink ref="C12" r:id="rId42"/>
+    <hyperlink ref="E12" r:id="rId43"/>
+    <hyperlink ref="H12" r:id="rId44"/>
+    <hyperlink ref="J12" r:id="rId45"/>
+    <hyperlink ref="C13" r:id="rId46"/>
+    <hyperlink ref="E13" r:id="rId47"/>
+    <hyperlink ref="H13" r:id="rId48"/>
+    <hyperlink ref="J13" r:id="rId49"/>
+    <hyperlink ref="C14" r:id="rId50"/>
+    <hyperlink ref="E14" r:id="rId51"/>
+    <hyperlink ref="H14" r:id="rId52"/>
+    <hyperlink ref="J14" r:id="rId53"/>
+    <hyperlink ref="C15" r:id="rId54"/>
+    <hyperlink ref="E15" r:id="rId55"/>
+    <hyperlink ref="H15" r:id="rId56"/>
+    <hyperlink ref="J15" r:id="rId57"/>
+    <hyperlink ref="C16" r:id="rId58"/>
+    <hyperlink ref="E16" r:id="rId59"/>
+    <hyperlink ref="H16" r:id="rId60"/>
+    <hyperlink ref="J16" r:id="rId61"/>
   </hyperlinks>
-  <drawing r:id="rId62"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>